<commit_message>
Revise Samsung proposal per Loretta's feedback
- Retitle exec summary plainly; remove one-pager framing and download button
- Add outputs section and day-one example prompts (what users actually get)
- Add joined-up analysis pipeline: inputs, analysis, outputs, decisions, MMM positioning
- Add use-cases-by-team section (Corporate Marketing, HEA, Mobile later)
- Name external sources: Sprinklr, Nielsen, Bloomberg, Meta, footfall providers
- Add future-fit section (no stranded cost, coexists with HQ AI plans)
- Convert close into three next steps incl. technical validation session
- Renumber sections, sync checklist, matrix workbook and both PDFs

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samsung-insights-engine/Samsung-Insights-Engine-Compliance-Matrix.xlsx
+++ b/samsung-insights-engine/Samsung-Insights-Engine-Compliance-Matrix.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="161">
   <si>
     <t xml:space="preserve">Samsung Insights Engine · Requirements Compliance Matrix</t>
   </si>
@@ -240,6 +240,15 @@
     <t xml:space="preserve">Architecturally fenced: no connector exists, no such content indexed</t>
   </si>
   <si>
+    <t xml:space="preserve">Ingest external data platforms Samsung licenses (Sprinklr, Nielsen, Bloomberg, Meta, footfall and local-market providers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As access granted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Via API, scheduled file transfer or cloud share; the Engine is agnostic to the source system</t>
+  </si>
+  <si>
     <t xml:space="preserve">Legend: Comply = capability available at deployment within the stated window. Comply - committed = capability contractually committed for delivery inside the brief's own phase window.</t>
   </si>
   <si>
@@ -372,6 +381,12 @@
     <t xml:space="preserve">Samsung retains the deployed application in its own cloud. If the vendor disappeared, the Engine keeps running where it is.</t>
   </si>
   <si>
+    <t xml:space="preserve">Future fit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A subscription, not a capital build: nothing stranded, coexists with or powers any future global platform via the headless API.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Required Response Items · Coverage</t>
   </si>
   <si>
@@ -399,7 +414,7 @@
     <t xml:space="preserve">Recommended MVP scope in Phase 1, and phasing and roadmap if different</t>
   </si>
   <si>
-    <t xml:space="preserve">Section 03 (compressed roadmap), Section 09 (pilot), Appendix A8</t>
+    <t xml:space="preserve">Section 03 (compressed roadmap), Section 10 (pilot), Appendix A8</t>
   </si>
   <si>
     <t xml:space="preserve">Data ingestion approach</t>
@@ -417,7 +432,7 @@
     <t xml:space="preserve">Security and permissions model</t>
   </si>
   <si>
-    <t xml:space="preserve">Section 06; Appendix A3</t>
+    <t xml:space="preserve">Section 07; Appendix A3</t>
   </si>
   <si>
     <t xml:space="preserve">AI model / RAG approach</t>
@@ -441,13 +456,13 @@
     <t xml:space="preserve">Example user experience</t>
   </si>
   <si>
-    <t xml:space="preserve">Interactive demonstration; Section 02</t>
+    <t xml:space="preserve">Interactive demonstration; Sections 02 and 06</t>
   </si>
   <si>
     <t xml:space="preserve">Any integration requirements</t>
   </si>
   <si>
-    <t xml:space="preserve">Appendix A6; Section 10</t>
+    <t xml:space="preserve">Appendix A6; Section 11</t>
   </si>
   <si>
     <t xml:space="preserve">Implementation timeline</t>
@@ -459,37 +474,37 @@
     <t xml:space="preserve">Cost estimate by phase</t>
   </si>
   <si>
-    <t xml:space="preserve">Section 08; Appendix A9; Commercials tab of this workbook</t>
+    <t xml:space="preserve">Section 09; Appendix A9; Commercials tab of this workbook</t>
   </si>
   <si>
     <t xml:space="preserve">Resource requirements from Samsung (BI, Marketing Ops, IT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Section 10; Appendix A8</t>
+    <t xml:space="preserve">Section 11; Appendix A8</t>
   </si>
   <si>
     <t xml:space="preserve">Risks and dependencies</t>
   </si>
   <si>
-    <t xml:space="preserve">Section 11</t>
+    <t xml:space="preserve">Section 12</t>
   </si>
   <si>
     <t xml:space="preserve">Pilot proposal</t>
   </si>
   <si>
-    <t xml:space="preserve">Section 09</t>
+    <t xml:space="preserve">Section 10</t>
   </si>
   <si>
     <t xml:space="preserve">Examples of relevant previous work</t>
   </si>
   <si>
-    <t xml:space="preserve">Section 07</t>
+    <t xml:space="preserve">Section 08</t>
   </si>
   <si>
     <t xml:space="preserve">Ongoing support model required</t>
   </si>
   <si>
-    <t xml:space="preserve">Section 08; Appendix A7</t>
+    <t xml:space="preserve">Section 09; Appendix A7</t>
   </si>
 </sst>
 </file>
@@ -974,7 +989,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1495,28 +1510,48 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="12" t="s">
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
+      <c r="C29" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="12" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
       <c r="E31" s="12"/>
       <c r="F31" s="12"/>
     </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B30:F30"/>
     <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1533,7 +1568,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -1544,125 +1579,125 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>10000</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>10000</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>15000</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B11" s="17" t="n">
         <f aca="false">B5+12*B6</f>
         <v>130000</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B12" s="17" t="n">
         <f aca="false">B5+12*B7</f>
         <v>190000</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1670,10 +1705,10 @@
         <v>11</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1681,10 +1716,10 @@
         <v>35</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1692,10 +1727,10 @@
         <v>49</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1703,58 +1738,69 @@
         <v>56</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C21" s="18"/>
       <c r="D21" s="18"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C22" s="18"/>
       <c r="D22" s="18"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C23" s="18"/>
       <c r="D23" s="18"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C24" s="18"/>
       <c r="D24" s="18"/>
     </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1782,12 +1828,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1795,13 +1841,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1809,13 +1855,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1823,13 +1869,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1837,13 +1883,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1851,13 +1897,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1865,13 +1911,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1879,13 +1925,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1893,13 +1939,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1907,13 +1953,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1921,13 +1967,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1935,13 +1981,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1949,13 +1995,13 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1963,13 +2009,13 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1977,13 +2023,13 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1991,13 +2037,13 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2005,13 +2051,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2019,13 +2065,13 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2033,13 +2079,13 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>